<commit_message>
feat ASP2103: add device logs reports
</commit_message>
<xml_diff>
--- a/api/templates/export/device_operation_logs/en.xlsx
+++ b/api/templates/export/device_operation_logs/en.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu-20.04\home\ubuntu\aspect\api\templates\export\device_operation_logs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF703F33-79C8-4D80-A2C7-6A0155851042}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="40" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAD53B1F-E053-4064-834C-D91399667930}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="40" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="480" yWindow="480" windowWidth="20730" windowHeight="11760" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -66,34 +66,34 @@
     <t>Text</t>
   </si>
   <si>
-    <t>&lt;errors&gt;</t>
-  </si>
-  <si>
-    <t>Errors</t>
-  </si>
-  <si>
     <t>Type</t>
   </si>
   <si>
     <t>&lt;logType&gt;</t>
   </si>
   <si>
-    <t>calibrations</t>
-  </si>
-  <si>
-    <t>&lt;calibrations&gt;</t>
-  </si>
-  <si>
-    <t>temperature</t>
-  </si>
-  <si>
     <t>&lt;temperature&gt;</t>
   </si>
   <si>
-    <t>voltage</t>
-  </si>
-  <si>
     <t>&lt;voltage&gt;</t>
+  </si>
+  <si>
+    <t>Temperature</t>
+  </si>
+  <si>
+    <t>Voltage</t>
+  </si>
+  <si>
+    <t>Calibration Message</t>
+  </si>
+  <si>
+    <t>&lt;calibrationMessage&gt;</t>
+  </si>
+  <si>
+    <t>Error Message</t>
+  </si>
+  <si>
+    <t>&lt;errorMessage&gt;</t>
   </si>
 </sst>
 </file>
@@ -103,7 +103,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]mmmm\ d\,\ yyyy;@"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -114,14 +114,6 @@
     <font>
       <b/>
       <sz val="12"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="16"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -146,6 +138,28 @@
     <font>
       <u/>
       <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="7"/>
+      <color rgb="FFCE9178"/>
+      <name val="Fira Code Retina"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="24"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -237,50 +251,50 @@
   </borders>
   <cellStyleXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -297,15 +311,12 @@
     <xf numFmtId="10" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -315,7 +326,13 @@
     <xf numFmtId="10" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -731,15 +748,16 @@
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="53.58203125" style="7" customWidth="1"/>
-    <col min="2" max="2" width="33.25" style="2" customWidth="1"/>
-    <col min="3" max="3" width="26.08203125" style="2" customWidth="1"/>
-    <col min="4" max="7" width="34.08203125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="26.08203125" style="2" customWidth="1"/>
+    <col min="3" max="4" width="34.08203125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="49" style="2" customWidth="1"/>
+    <col min="6" max="7" width="34.08203125" style="2" customWidth="1"/>
     <col min="8" max="8" width="67.58203125" style="2" customWidth="1"/>
-    <col min="9" max="9" width="56.08203125" style="2" customWidth="1"/>
+    <col min="9" max="9" width="33.25" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="21" x14ac:dyDescent="0.5">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:9" ht="31" x14ac:dyDescent="0.7">
+      <c r="A1" s="12" t="s">
         <v>2</v>
       </c>
     </row>
@@ -748,13 +766,13 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:9" s="7" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="12" t="s">
+    <row r="3" spans="1:9" s="7" customFormat="1" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A3" s="13" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:9" s="7" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="12" t="s">
+    <row r="4" spans="1:9" s="7" customFormat="1" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4" s="13" t="s">
         <v>4</v>
       </c>
     </row>
@@ -765,71 +783,71 @@
       </c>
     </row>
     <row r="7" spans="1:9" s="3" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="9" t="s">
+      <c r="A7" s="8" t="s">
         <v>5</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E7" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F7" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F7" s="1" t="s">
-        <v>19</v>
-      </c>
       <c r="G7" s="1" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="H7" s="1" t="s">
         <v>12</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C8" s="5" t="s">
+      <c r="B8" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D8" s="11" t="s">
+      <c r="C8" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="F8" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="G8" s="10" t="s">
         <v>16</v>
-      </c>
-      <c r="E8" s="11" t="s">
-        <v>18</v>
-      </c>
-      <c r="F8" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="G8" s="11" t="s">
-        <v>22</v>
       </c>
       <c r="H8" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="I8" s="11" t="s">
-        <v>13</v>
+      <c r="I8" s="4" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="B10" s="6"/>
       <c r="C10" s="6"/>
       <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
+      <c r="E10" s="11"/>
       <c r="F10" s="6"/>
       <c r="G10" s="6"/>
       <c r="H10" s="6"/>
-      <c r="I10" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fixing seeds, templates and report service.
</commit_message>
<xml_diff>
--- a/api/templates/export/device_operation_logs/en.xlsx
+++ b/api/templates/export/device_operation_logs/en.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu-20.04\home\ubuntu\aspect\api\templates\export\device_operation_logs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAD53B1F-E053-4064-834C-D91399667930}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="40" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0FA055F-FDE5-4B8C-A30E-B84D30C0A139}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="40" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="480" yWindow="480" windowWidth="20730" windowHeight="11760" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>&lt;Table&gt;</t>
   </si>
@@ -60,40 +60,16 @@
     <t>&lt;logLevel&gt;</t>
   </si>
   <si>
-    <t>&lt;logText&gt;</t>
-  </si>
-  <si>
-    <t>Text</t>
-  </si>
-  <si>
     <t>Type</t>
   </si>
   <si>
     <t>&lt;logType&gt;</t>
   </si>
   <si>
-    <t>&lt;temperature&gt;</t>
-  </si>
-  <si>
-    <t>&lt;voltage&gt;</t>
-  </si>
-  <si>
-    <t>Temperature</t>
-  </si>
-  <si>
-    <t>Voltage</t>
-  </si>
-  <si>
-    <t>Calibration Message</t>
-  </si>
-  <si>
-    <t>&lt;calibrationMessage&gt;</t>
-  </si>
-  <si>
-    <t>Error Message</t>
-  </si>
-  <si>
-    <t>&lt;errorMessage&gt;</t>
+    <t>Message</t>
+  </si>
+  <si>
+    <t>&lt;message&gt;</t>
   </si>
 </sst>
 </file>
@@ -294,7 +270,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -305,9 +281,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -334,6 +307,15 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="43">
@@ -744,110 +726,80 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="53.58203125" style="7" customWidth="1"/>
-    <col min="2" max="2" width="26.08203125" style="2" customWidth="1"/>
-    <col min="3" max="4" width="34.08203125" style="2" customWidth="1"/>
-    <col min="5" max="5" width="49" style="2" customWidth="1"/>
-    <col min="6" max="7" width="34.08203125" style="2" customWidth="1"/>
-    <col min="8" max="8" width="67.58203125" style="2" customWidth="1"/>
-    <col min="9" max="9" width="33.25" style="2" customWidth="1"/>
+    <col min="1" max="1" width="14.9140625" style="6" customWidth="1"/>
+    <col min="2" max="2" width="17.25" style="2" customWidth="1"/>
+    <col min="3" max="3" width="14.4140625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="79.83203125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="122.5" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="31" x14ac:dyDescent="0.7">
-      <c r="A1" s="12" t="s">
+    <row r="1" spans="1:5" ht="31" x14ac:dyDescent="0.7">
+      <c r="A1" s="11" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:9" s="7" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="7" t="s">
+    <row r="2" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="6" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:9" s="7" customFormat="1" ht="23.5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A3" s="13" t="s">
+    <row r="3" spans="1:5" s="6" customFormat="1" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A3" s="12" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:9" s="7" customFormat="1" ht="23.5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A4" s="13" t="s">
+    <row r="4" spans="1:5" s="6" customFormat="1" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4" s="12" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:9" s="7" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="6" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="7" t="s">
+    <row r="5" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="6" spans="1:5" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="6" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:9" s="3" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="8" t="s">
+    <row r="7" spans="1:5" s="3" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="7" t="s">
         <v>5</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C7" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="H7" s="1" t="s">
+      <c r="E7" s="15" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="I7" s="1" t="s">
-        <v>7</v>
+      <c r="D8" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" s="13" t="s">
+        <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="C8" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="D8" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="E8" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="F8" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="G8" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="H8" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="I8" s="4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="B10" s="6"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="11"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
-      <c r="H10" s="6"/>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B10" s="5"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>